<commit_message>
feat(meet): add 18 cash expense entries to meet account and synchronize database, stores and excel
</commit_message>
<xml_diff>
--- a/Expense_Entries_Date_Wise.xlsx
+++ b/Expense_Entries_Date_Wise.xlsx
@@ -5,13 +5,14 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Expenses" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Meet Cash Expenses" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="196">
   <si>
     <t>Entry ID</t>
   </si>
@@ -203,13 +204,412 @@
   </si>
   <si>
     <t>Original entry had no date; included in total.</t>
+  </si>
+  <si>
+    <t>Dal makhani</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 1 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>23/09</t>
+  </si>
+  <si>
+    <t>Rajnigandha</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 2 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Frido orders</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 3 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Amzone</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 4 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>28/09</t>
+  </si>
+  <si>
+    <t>Pizaa olio and</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 5 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Amzone pay add money</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 6 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>30/09</t>
+  </si>
+  <si>
+    <t>Cash Amzone cell charger</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 7 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Defender Number Plat charge</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 8 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>02/10</t>
+  </si>
+  <si>
+    <t>Defender</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 9 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 10 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Amzone cell order</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 11 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Bhabhi order parcel</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 12 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 13 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Dal makhani saman</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 14 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>08/10</t>
+  </si>
+  <si>
+    <t>Home pizaa items</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 15 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Amzone home</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 16 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 17 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Medicine tharmomitsr</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. 18 - Added for Meet (Payment: Cash)</t>
+  </si>
+  <si>
+    <t>Sr.</t>
+  </si>
+  <si>
+    <t>Date (DD/MM/YY)</t>
+  </si>
+  <si>
+    <t>Expense Date</t>
+  </si>
+  <si>
+    <t>Expense ID</t>
+  </si>
+  <si>
+    <t>Description / Title</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
+  </si>
+  <si>
+    <t>User Account</t>
+  </si>
+  <si>
+    <t>Vendor</t>
+  </si>
+  <si>
+    <t>21/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-21</t>
+  </si>
+  <si>
+    <t>EXP-20260921-MC01</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>Meet</t>
+  </si>
+  <si>
+    <t>Dal Makhani</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 1 - Added for Meet</t>
+  </si>
+  <si>
+    <t>23/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-23</t>
+  </si>
+  <si>
+    <t>EXP-20260923-MC02</t>
+  </si>
+  <si>
+    <t>Miscellaneous</t>
+  </si>
+  <si>
+    <t>Local Store</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 2 - Added for Meet</t>
+  </si>
+  <si>
+    <t>25/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
+  </si>
+  <si>
+    <t>EXP-20260925-MC03</t>
+  </si>
+  <si>
+    <t>Shopping</t>
+  </si>
+  <si>
+    <t>Frido</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 3 - Added for Meet</t>
+  </si>
+  <si>
+    <t>27/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>EXP-20260927-MC04</t>
+  </si>
+  <si>
+    <t>Amazon</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 4 - Added for Meet</t>
+  </si>
+  <si>
+    <t>28/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>EXP-20260928-MC05</t>
+  </si>
+  <si>
+    <t>Olio Pizza</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 5 - Added for Meet</t>
+  </si>
+  <si>
+    <t>EXP-20260928-MC06</t>
+  </si>
+  <si>
+    <t>Amazon Pay</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 6 - Added for Meet</t>
+  </si>
+  <si>
+    <t>30/09/26</t>
+  </si>
+  <si>
+    <t>2026-09-30</t>
+  </si>
+  <si>
+    <t>EXP-20260930-MC07</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 7 - Added for Meet</t>
+  </si>
+  <si>
+    <t>01/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>EXP-20261001-MC08</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Defender RTO / Number Plate Vendor</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 8 - Added for Meet</t>
+  </si>
+  <si>
+    <t>02/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>EXP-20261002-MC09</t>
+  </si>
+  <si>
+    <t>Defender Service</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 9 - Added for Meet</t>
+  </si>
+  <si>
+    <t>EXP-20261002-MC10</t>
+  </si>
+  <si>
+    <t>Mahakali Dhaba</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 10 - Added for Meet</t>
+  </si>
+  <si>
+    <t>EXP-20261002-MC11</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 11 - Added for Meet</t>
+  </si>
+  <si>
+    <t>04/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>EXP-20261004-MC12</t>
+  </si>
+  <si>
+    <t>Parcel Delivery / Store</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 12 - Added for Meet</t>
+  </si>
+  <si>
+    <t>EXP-20261004-MC13</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 13 - Added for Meet</t>
+  </si>
+  <si>
+    <t>05/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-05</t>
+  </si>
+  <si>
+    <t>EXP-20261005-MC14</t>
+  </si>
+  <si>
+    <t>Grocery</t>
+  </si>
+  <si>
+    <t>Grocery Store</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 14 - Added for Meet</t>
+  </si>
+  <si>
+    <t>08/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>EXP-20261008-MC15</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 15 - Added for Meet</t>
+  </si>
+  <si>
+    <t>12/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-12</t>
+  </si>
+  <si>
+    <t>EXP-20261012-MC16</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 16 - Added for Meet</t>
+  </si>
+  <si>
+    <t>19/10/26</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>EXP-20261019-MC17</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 17 - Added for Meet</t>
+  </si>
+  <si>
+    <t>EXP-20261019-MC18</t>
+  </si>
+  <si>
+    <t>Medical</t>
+  </si>
+  <si>
+    <t>Pharmacy / Medical Store</t>
+  </si>
+  <si>
+    <t>Cash Entry Sr. No. 18 - Added for Meet</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Total 18 Cash Expenses</t>
+  </si>
+  <si>
+    <t>Sum of all 18 Cash entries</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="₹#,##0"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -217,13 +617,25 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E293B"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -238,8 +650,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +995,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1230,6 +1646,1089 @@
         <v>63</v>
       </c>
     </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>25</v>
+      </c>
+      <c r="D33" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33">
+        <v>1200</v>
+      </c>
+      <c r="F33" t="s">
+        <v>8</v>
+      </c>
+      <c r="G33" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>33</v>
+      </c>
+      <c r="C34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" t="s">
+        <v>67</v>
+      </c>
+      <c r="E34">
+        <v>420</v>
+      </c>
+      <c r="F34" t="s">
+        <v>8</v>
+      </c>
+      <c r="G34" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>34</v>
+      </c>
+      <c r="C35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D35" t="s">
+        <v>69</v>
+      </c>
+      <c r="E35">
+        <v>3000</v>
+      </c>
+      <c r="F35" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>35</v>
+      </c>
+      <c r="C36" t="s">
+        <v>35</v>
+      </c>
+      <c r="D36" t="s">
+        <v>71</v>
+      </c>
+      <c r="E36">
+        <v>700</v>
+      </c>
+      <c r="F36" t="s">
+        <v>8</v>
+      </c>
+      <c r="G36" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>36</v>
+      </c>
+      <c r="C37" t="s">
+        <v>73</v>
+      </c>
+      <c r="D37" t="s">
+        <v>74</v>
+      </c>
+      <c r="E37">
+        <v>900</v>
+      </c>
+      <c r="F37" t="s">
+        <v>8</v>
+      </c>
+      <c r="G37" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>37</v>
+      </c>
+      <c r="C38" t="s">
+        <v>73</v>
+      </c>
+      <c r="D38" t="s">
+        <v>76</v>
+      </c>
+      <c r="E38">
+        <v>1500</v>
+      </c>
+      <c r="F38" t="s">
+        <v>8</v>
+      </c>
+      <c r="G38" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>38</v>
+      </c>
+      <c r="C39" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39" t="s">
+        <v>79</v>
+      </c>
+      <c r="E39">
+        <v>1450</v>
+      </c>
+      <c r="F39" t="s">
+        <v>8</v>
+      </c>
+      <c r="G39" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>39</v>
+      </c>
+      <c r="C40" t="s">
+        <v>39</v>
+      </c>
+      <c r="D40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E40">
+        <v>500</v>
+      </c>
+      <c r="F40" t="s">
+        <v>8</v>
+      </c>
+      <c r="G40" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B41">
+        <v>40</v>
+      </c>
+      <c r="C41" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41">
+        <v>1200</v>
+      </c>
+      <c r="F41" t="s">
+        <v>8</v>
+      </c>
+      <c r="G41" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>41</v>
+      </c>
+      <c r="C42" t="s">
+        <v>83</v>
+      </c>
+      <c r="D42" t="s">
+        <v>61</v>
+      </c>
+      <c r="E42">
+        <v>5000</v>
+      </c>
+      <c r="F42" t="s">
+        <v>8</v>
+      </c>
+      <c r="G42" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>42</v>
+      </c>
+      <c r="C43" t="s">
+        <v>83</v>
+      </c>
+      <c r="D43" t="s">
+        <v>87</v>
+      </c>
+      <c r="E43">
+        <v>1200</v>
+      </c>
+      <c r="F43" t="s">
+        <v>8</v>
+      </c>
+      <c r="G43" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>43</v>
+      </c>
+      <c r="C44" t="s">
+        <v>42</v>
+      </c>
+      <c r="D44" t="s">
+        <v>89</v>
+      </c>
+      <c r="E44">
+        <v>1700</v>
+      </c>
+      <c r="F44" t="s">
+        <v>8</v>
+      </c>
+      <c r="G44" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>44</v>
+      </c>
+      <c r="C45" t="s">
+        <v>42</v>
+      </c>
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45">
+        <v>500</v>
+      </c>
+      <c r="F45" t="s">
+        <v>8</v>
+      </c>
+      <c r="G45" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>44</v>
+      </c>
+      <c r="D46" t="s">
+        <v>92</v>
+      </c>
+      <c r="E46">
+        <v>1700</v>
+      </c>
+      <c r="F46" t="s">
+        <v>8</v>
+      </c>
+      <c r="G46" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>46</v>
+      </c>
+      <c r="C47" t="s">
+        <v>94</v>
+      </c>
+      <c r="D47" t="s">
+        <v>95</v>
+      </c>
+      <c r="E47">
+        <v>1800</v>
+      </c>
+      <c r="F47" t="s">
+        <v>8</v>
+      </c>
+      <c r="G47" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B48">
+        <v>47</v>
+      </c>
+      <c r="C48" t="s">
+        <v>52</v>
+      </c>
+      <c r="D48" t="s">
+        <v>97</v>
+      </c>
+      <c r="E48">
+        <v>1500</v>
+      </c>
+      <c r="F48" t="s">
+        <v>8</v>
+      </c>
+      <c r="G48" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>48</v>
+      </c>
+      <c r="C49" t="s">
+        <v>58</v>
+      </c>
+      <c r="D49" t="s">
+        <v>18</v>
+      </c>
+      <c r="E49">
+        <v>700</v>
+      </c>
+      <c r="F49" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>49</v>
+      </c>
+      <c r="C50" t="s">
+        <v>58</v>
+      </c>
+      <c r="D50" t="s">
+        <v>100</v>
+      </c>
+      <c r="E50">
+        <v>2000</v>
+      </c>
+      <c r="F50" t="s">
+        <v>8</v>
+      </c>
+      <c r="G50" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="10" max="10" width="25" customWidth="1"/>
+    <col min="11" max="11" width="35" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1200</v>
+      </c>
+      <c r="H2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J2" t="s">
+        <v>117</v>
+      </c>
+      <c r="K2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" t="s">
+        <v>122</v>
+      </c>
+      <c r="G3" s="2">
+        <v>420</v>
+      </c>
+      <c r="H3" t="s">
+        <v>115</v>
+      </c>
+      <c r="I3" t="s">
+        <v>116</v>
+      </c>
+      <c r="J3" t="s">
+        <v>123</v>
+      </c>
+      <c r="K3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" t="s">
+        <v>128</v>
+      </c>
+      <c r="G4" s="2">
+        <v>3000</v>
+      </c>
+      <c r="H4" t="s">
+        <v>115</v>
+      </c>
+      <c r="I4" t="s">
+        <v>116</v>
+      </c>
+      <c r="J4" t="s">
+        <v>129</v>
+      </c>
+      <c r="K4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G5" s="2">
+        <v>700</v>
+      </c>
+      <c r="H5" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" t="s">
+        <v>116</v>
+      </c>
+      <c r="J5" t="s">
+        <v>134</v>
+      </c>
+      <c r="K5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D6" t="s">
+        <v>138</v>
+      </c>
+      <c r="E6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" s="2">
+        <v>900</v>
+      </c>
+      <c r="H6" t="s">
+        <v>115</v>
+      </c>
+      <c r="I6" t="s">
+        <v>116</v>
+      </c>
+      <c r="J6" t="s">
+        <v>139</v>
+      </c>
+      <c r="K6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F7" t="s">
+        <v>122</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1500</v>
+      </c>
+      <c r="H7" t="s">
+        <v>115</v>
+      </c>
+      <c r="I7" t="s">
+        <v>116</v>
+      </c>
+      <c r="J7" t="s">
+        <v>142</v>
+      </c>
+      <c r="K7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" t="s">
+        <v>145</v>
+      </c>
+      <c r="D8" t="s">
+        <v>146</v>
+      </c>
+      <c r="E8" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" t="s">
+        <v>128</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1450</v>
+      </c>
+      <c r="H8" t="s">
+        <v>115</v>
+      </c>
+      <c r="I8" t="s">
+        <v>116</v>
+      </c>
+      <c r="J8" t="s">
+        <v>134</v>
+      </c>
+      <c r="K8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D9" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G9" s="2">
+        <v>500</v>
+      </c>
+      <c r="H9" t="s">
+        <v>115</v>
+      </c>
+      <c r="I9" t="s">
+        <v>116</v>
+      </c>
+      <c r="J9" t="s">
+        <v>152</v>
+      </c>
+      <c r="K9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D10" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" t="s">
+        <v>151</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1200</v>
+      </c>
+      <c r="H10" t="s">
+        <v>115</v>
+      </c>
+      <c r="I10" t="s">
+        <v>116</v>
+      </c>
+      <c r="J10" t="s">
+        <v>157</v>
+      </c>
+      <c r="K10" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G11" s="2">
+        <v>5000</v>
+      </c>
+      <c r="H11" t="s">
+        <v>115</v>
+      </c>
+      <c r="I11" t="s">
+        <v>116</v>
+      </c>
+      <c r="J11" t="s">
+        <v>160</v>
+      </c>
+      <c r="K11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>154</v>
+      </c>
+      <c r="C12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" t="s">
+        <v>87</v>
+      </c>
+      <c r="F12" t="s">
+        <v>128</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1200</v>
+      </c>
+      <c r="H12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" t="s">
+        <v>116</v>
+      </c>
+      <c r="J12" t="s">
+        <v>134</v>
+      </c>
+      <c r="K12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" t="s">
+        <v>165</v>
+      </c>
+      <c r="D13" t="s">
+        <v>166</v>
+      </c>
+      <c r="E13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F13" t="s">
+        <v>128</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1700</v>
+      </c>
+      <c r="H13" t="s">
+        <v>115</v>
+      </c>
+      <c r="I13" t="s">
+        <v>116</v>
+      </c>
+      <c r="J13" t="s">
+        <v>167</v>
+      </c>
+      <c r="K13" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D14" t="s">
+        <v>169</v>
+      </c>
+      <c r="E14" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s">
+        <v>128</v>
+      </c>
+      <c r="G14" s="2">
+        <v>500</v>
+      </c>
+      <c r="H14" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" t="s">
+        <v>116</v>
+      </c>
+      <c r="J14" t="s">
+        <v>123</v>
+      </c>
+      <c r="K14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" t="s">
+        <v>172</v>
+      </c>
+      <c r="D15" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" t="s">
+        <v>174</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1700</v>
+      </c>
+      <c r="H15" t="s">
+        <v>115</v>
+      </c>
+      <c r="I15" t="s">
+        <v>116</v>
+      </c>
+      <c r="J15" t="s">
+        <v>175</v>
+      </c>
+      <c r="K15" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" t="s">
+        <v>178</v>
+      </c>
+      <c r="D16" t="s">
+        <v>179</v>
+      </c>
+      <c r="E16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F16" t="s">
+        <v>174</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1800</v>
+      </c>
+      <c r="H16" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" t="s">
+        <v>116</v>
+      </c>
+      <c r="J16" t="s">
+        <v>175</v>
+      </c>
+      <c r="K16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>181</v>
+      </c>
+      <c r="C17" t="s">
+        <v>182</v>
+      </c>
+      <c r="D17" t="s">
+        <v>183</v>
+      </c>
+      <c r="E17" t="s">
+        <v>97</v>
+      </c>
+      <c r="F17" t="s">
+        <v>128</v>
+      </c>
+      <c r="G17" s="2">
+        <v>1500</v>
+      </c>
+      <c r="H17" t="s">
+        <v>115</v>
+      </c>
+      <c r="I17" t="s">
+        <v>116</v>
+      </c>
+      <c r="J17" t="s">
+        <v>134</v>
+      </c>
+      <c r="K17" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>185</v>
+      </c>
+      <c r="C18" t="s">
+        <v>186</v>
+      </c>
+      <c r="D18" t="s">
+        <v>187</v>
+      </c>
+      <c r="E18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" t="s">
+        <v>174</v>
+      </c>
+      <c r="G18" s="2">
+        <v>700</v>
+      </c>
+      <c r="H18" t="s">
+        <v>115</v>
+      </c>
+      <c r="I18" t="s">
+        <v>116</v>
+      </c>
+      <c r="J18" t="s">
+        <v>18</v>
+      </c>
+      <c r="K18" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D19" t="s">
+        <v>189</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
+      </c>
+      <c r="F19" t="s">
+        <v>190</v>
+      </c>
+      <c r="G19" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H19" t="s">
+        <v>115</v>
+      </c>
+      <c r="I19" t="s">
+        <v>116</v>
+      </c>
+      <c r="J19" t="s">
+        <v>191</v>
+      </c>
+      <c r="K19" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" s="4">
+        <v>26970</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>